<commit_message>
Publish LaSeu_2019_WWC, LaSeu_2021_WC, LaSeu_2022_WC, LaSeu_2023_WC
</commit_message>
<xml_diff>
--- a/events/LaSeu_2019_WWC/LaSeu_2019_WWC_start.xlsx
+++ b/events/LaSeu_2019_WWC/LaSeu_2019_WWC_start.xlsx
@@ -3709,6 +3709,11 @@
           <t>35512</t>
         </is>
       </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>35516</t>
+        </is>
+      </c>
       <c r="AC35" t="inlineStr">
         <is>
           <t>43076</t>

</xml_diff>